<commit_message>
Respaldo automático: 2026-09-11 09:02
</commit_message>
<xml_diff>
--- a/NotasPrimerCorte.xlsx
+++ b/NotasPrimerCorte.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10503"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/unicordoba/Documents/Cursos/Computacional/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0FF8C84C-A082-374F-BC3F-53967EDC380E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CAF9C80-0976-F645-896B-5F7ED57F4C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -239,7 +239,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -252,8 +252,20 @@
         <bgColor rgb="FF99CCFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -356,12 +368,59 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -374,40 +433,20 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -712,7 +751,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
@@ -723,59 +762,55 @@
     <col min="7" max="7" width="5.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="11"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="11"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="1"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="11"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="1"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="B4" s="9"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="10"/>
-      <c r="I4" s="11"/>
-    </row>
-    <row r="5" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="16"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="1"/>
+    </row>
+    <row r="5" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>58</v>
       </c>
@@ -785,597 +820,662 @@
       <c r="E5" s="7"/>
       <c r="F5" s="7"/>
       <c r="G5" s="8"/>
-      <c r="H5" s="10"/>
-      <c r="I5" s="11"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A6" s="13" t="s">
+      <c r="H5" s="1"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B6" s="14"/>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="11"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A7" s="16" t="s">
-        <v>0</v>
-      </c>
-      <c r="B7" s="16" t="s">
-        <v>1</v>
-      </c>
-      <c r="C7" s="17" t="s">
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="2"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="D7" s="17" t="s">
+      <c r="D7" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="F7" s="17" t="s">
+      <c r="F7" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="G7" s="17" t="s">
+      <c r="G7" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A8" s="16" t="s">
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="18">
+      <c r="C8" s="5">
         <v>0.91</v>
       </c>
-      <c r="D8" s="18">
+      <c r="D8" s="5">
         <v>2.5</v>
       </c>
-      <c r="E8" s="18">
-        <v>5</v>
-      </c>
-      <c r="F8" s="18">
-        <v>5</v>
-      </c>
-      <c r="G8" s="18">
+      <c r="E8" s="5">
+        <v>5</v>
+      </c>
+      <c r="F8" s="5">
+        <v>5</v>
+      </c>
+      <c r="G8" s="5">
         <f>C8*0.4+D8*0.3+E8*0.15+F8*0.15</f>
         <v>2.6139999999999999</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A9" s="16" t="s">
+      <c r="H8" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A9" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="16" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" s="18">
-        <v>0</v>
-      </c>
-      <c r="D9" s="18">
+      <c r="B9" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="19">
+        <v>5</v>
+      </c>
+      <c r="D9" s="19">
         <v>4.18</v>
       </c>
-      <c r="E9" s="18">
-        <v>5</v>
-      </c>
-      <c r="F9" s="18">
+      <c r="E9" s="19">
+        <v>5</v>
+      </c>
+      <c r="F9" s="19">
         <v>4.5999999999999996</v>
       </c>
-      <c r="G9" s="18">
+      <c r="G9" s="19">
         <f t="shared" ref="G9:G30" si="0">C9*0.4+D9*0.3+E9*0.15+F9*0.15</f>
-        <v>2.6939999999999995</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A10" s="16" t="s">
+        <v>4.6939999999999991</v>
+      </c>
+      <c r="H9" s="21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="18">
+      <c r="C10" s="5">
         <v>4.7699999999999996</v>
       </c>
-      <c r="D10" s="18">
+      <c r="D10" s="5">
         <v>4.97</v>
       </c>
-      <c r="E10" s="18">
-        <v>5</v>
-      </c>
-      <c r="F10" s="18">
-        <v>5</v>
-      </c>
-      <c r="G10" s="18">
+      <c r="E10" s="5">
+        <v>5</v>
+      </c>
+      <c r="F10" s="5">
+        <v>5</v>
+      </c>
+      <c r="G10" s="5">
         <f t="shared" si="0"/>
         <v>4.899</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A11" s="16" t="s">
+      <c r="H10" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="18">
+      <c r="C11" s="5">
         <v>1.36</v>
       </c>
-      <c r="D11" s="18">
+      <c r="D11" s="5">
         <v>4.87</v>
       </c>
-      <c r="E11" s="18">
-        <v>5</v>
-      </c>
-      <c r="F11" s="18">
-        <v>5</v>
-      </c>
-      <c r="G11" s="18">
+      <c r="E11" s="5">
+        <v>5</v>
+      </c>
+      <c r="F11" s="5">
+        <v>5</v>
+      </c>
+      <c r="G11" s="5">
         <f t="shared" si="0"/>
         <v>3.5049999999999999</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12" s="16" t="s">
+      <c r="H11" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="16" t="s">
+      <c r="B12" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="18">
+      <c r="C12" s="5">
         <v>3.86</v>
       </c>
-      <c r="D12" s="18">
+      <c r="D12" s="5">
         <v>1.35</v>
       </c>
-      <c r="E12" s="18">
-        <v>5</v>
-      </c>
-      <c r="F12" s="18">
-        <v>5</v>
-      </c>
-      <c r="G12" s="18">
+      <c r="E12" s="5">
+        <v>5</v>
+      </c>
+      <c r="F12" s="5">
+        <v>5</v>
+      </c>
+      <c r="G12" s="5">
         <f t="shared" si="0"/>
         <v>3.4489999999999998</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13" s="16" t="s">
+      <c r="H12" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A13" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="16" t="s">
+      <c r="B13" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="18">
-        <v>0</v>
-      </c>
-      <c r="D13" s="18">
-        <v>0</v>
-      </c>
-      <c r="E13" s="18">
-        <v>0</v>
-      </c>
-      <c r="F13" s="18">
-        <v>5</v>
-      </c>
-      <c r="G13" s="18">
+      <c r="C13" s="24">
+        <v>0</v>
+      </c>
+      <c r="D13" s="24">
+        <v>0</v>
+      </c>
+      <c r="E13" s="24">
+        <v>0</v>
+      </c>
+      <c r="F13" s="24">
+        <v>5</v>
+      </c>
+      <c r="G13" s="24">
         <f t="shared" si="0"/>
         <v>0.75</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A14" s="16" t="s">
+      <c r="H13" s="25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A14" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="16" t="s">
+      <c r="B14" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="18">
-        <v>5</v>
-      </c>
-      <c r="D14" s="18">
+      <c r="C14" s="5">
+        <v>5</v>
+      </c>
+      <c r="D14" s="5">
         <v>4.51</v>
       </c>
-      <c r="E14" s="18">
-        <v>5</v>
-      </c>
-      <c r="F14" s="18">
-        <v>5</v>
-      </c>
-      <c r="G14" s="18">
+      <c r="E14" s="5">
+        <v>5</v>
+      </c>
+      <c r="F14" s="5">
+        <v>5</v>
+      </c>
+      <c r="G14" s="5">
         <f t="shared" si="0"/>
         <v>4.8529999999999998</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A15" s="16" t="s">
+      <c r="H14" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A15" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="16" t="s">
+      <c r="B15" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C15" s="18">
+      <c r="C15" s="5">
         <v>3.18</v>
       </c>
-      <c r="D15" s="18">
+      <c r="D15" s="5">
         <v>2.44</v>
       </c>
-      <c r="E15" s="18">
-        <v>0</v>
-      </c>
-      <c r="F15" s="18">
-        <v>5</v>
-      </c>
-      <c r="G15" s="18">
+      <c r="E15" s="5">
+        <v>0</v>
+      </c>
+      <c r="F15" s="5">
+        <v>5</v>
+      </c>
+      <c r="G15" s="5">
         <f t="shared" si="0"/>
         <v>2.7540000000000004</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A16" s="16" t="s">
+      <c r="H15" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="16" t="s">
+      <c r="B16" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="18">
+      <c r="C16" s="5">
         <v>1.36</v>
       </c>
-      <c r="D16" s="18">
+      <c r="D16" s="5">
         <v>1.1399999999999999</v>
       </c>
-      <c r="E16" s="18">
-        <v>5</v>
-      </c>
-      <c r="F16" s="18">
+      <c r="E16" s="5">
+        <v>5</v>
+      </c>
+      <c r="F16" s="5">
         <v>4.5</v>
       </c>
-      <c r="G16" s="18">
+      <c r="G16" s="5">
         <f t="shared" si="0"/>
         <v>2.3109999999999999</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A17" s="16" t="s">
+      <c r="H16" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="18">
-        <v>0</v>
-      </c>
-      <c r="D17" s="18">
-        <v>0</v>
-      </c>
-      <c r="E17" s="18">
-        <v>0</v>
-      </c>
-      <c r="F17" s="18">
+      <c r="C17" s="5">
+        <v>0</v>
+      </c>
+      <c r="D17" s="5">
+        <v>0</v>
+      </c>
+      <c r="E17" s="5">
+        <v>0</v>
+      </c>
+      <c r="F17" s="5">
         <v>4.5</v>
       </c>
-      <c r="G17" s="18">
+      <c r="G17" s="5">
         <f t="shared" si="0"/>
         <v>0.67499999999999993</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A18" s="16" t="s">
+      <c r="H17" s="22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="16" t="s">
+      <c r="B18" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="18">
+      <c r="C18" s="5">
         <v>4.09</v>
       </c>
-      <c r="D18" s="18">
+      <c r="D18" s="5">
         <v>3.27</v>
       </c>
-      <c r="E18" s="18">
-        <v>0</v>
-      </c>
-      <c r="F18" s="18">
-        <v>5</v>
-      </c>
-      <c r="G18" s="18">
+      <c r="E18" s="5">
+        <v>0</v>
+      </c>
+      <c r="F18" s="5">
+        <v>5</v>
+      </c>
+      <c r="G18" s="5">
         <f t="shared" si="0"/>
         <v>3.367</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A19" s="16" t="s">
+      <c r="H18" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="16" t="s">
+      <c r="B19" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="18">
+      <c r="C19" s="5">
         <v>4.09</v>
       </c>
-      <c r="D19" s="18">
+      <c r="D19" s="5">
         <v>4.17</v>
       </c>
-      <c r="E19" s="18">
-        <v>0</v>
-      </c>
-      <c r="F19" s="18">
-        <v>5</v>
-      </c>
-      <c r="G19" s="18">
+      <c r="E19" s="5">
+        <v>0</v>
+      </c>
+      <c r="F19" s="5">
+        <v>5</v>
+      </c>
+      <c r="G19" s="5">
         <f t="shared" si="0"/>
         <v>3.637</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A20" s="16" t="s">
+      <c r="H19" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="16" t="s">
+      <c r="B20" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C20" s="18">
+      <c r="C20" s="5">
         <v>3.86</v>
       </c>
-      <c r="D20" s="18">
+      <c r="D20" s="5">
         <v>3.33</v>
       </c>
-      <c r="E20" s="18">
-        <v>0</v>
-      </c>
-      <c r="F20" s="18">
-        <v>5</v>
-      </c>
-      <c r="G20" s="18">
+      <c r="E20" s="5">
+        <v>0</v>
+      </c>
+      <c r="F20" s="5">
+        <v>5</v>
+      </c>
+      <c r="G20" s="5">
         <f t="shared" si="0"/>
         <v>3.2930000000000001</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A21" s="16" t="s">
+      <c r="H20" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A21" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="16" t="s">
+      <c r="B21" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C21" s="18">
+      <c r="C21" s="5">
         <v>4.7699999999999996</v>
       </c>
-      <c r="D21" s="18">
+      <c r="D21" s="5">
         <v>4.0999999999999996</v>
       </c>
-      <c r="E21" s="18">
-        <v>5</v>
-      </c>
-      <c r="F21" s="18">
-        <v>5</v>
-      </c>
-      <c r="G21" s="18">
+      <c r="E21" s="5">
+        <v>5</v>
+      </c>
+      <c r="F21" s="5">
+        <v>5</v>
+      </c>
+      <c r="G21" s="5">
         <f t="shared" si="0"/>
         <v>4.6379999999999999</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A22" s="16" t="s">
+      <c r="H21" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A22" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="B22" s="16" t="s">
+      <c r="B22" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="C22" s="18">
-        <v>0</v>
-      </c>
-      <c r="D22" s="18">
+      <c r="C22" s="19">
+        <v>5</v>
+      </c>
+      <c r="D22" s="19">
         <v>4.46</v>
       </c>
-      <c r="E22" s="18">
-        <v>0</v>
-      </c>
-      <c r="F22" s="18">
-        <v>5</v>
-      </c>
-      <c r="G22" s="18">
-        <f t="shared" si="0"/>
-        <v>2.0880000000000001</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A23" s="16" t="s">
+      <c r="E22" s="19">
+        <v>0</v>
+      </c>
+      <c r="F22" s="19">
+        <v>5</v>
+      </c>
+      <c r="G22" s="19">
+        <f t="shared" si="0"/>
+        <v>4.0880000000000001</v>
+      </c>
+      <c r="H22" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B23" s="16" t="s">
+      <c r="B23" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C23" s="18">
+      <c r="C23" s="5">
         <v>4.09</v>
       </c>
-      <c r="D23" s="18">
+      <c r="D23" s="5">
         <v>3.65</v>
       </c>
-      <c r="E23" s="18">
-        <v>5</v>
-      </c>
-      <c r="F23" s="18">
-        <v>5</v>
-      </c>
-      <c r="G23" s="18">
+      <c r="E23" s="5">
+        <v>5</v>
+      </c>
+      <c r="F23" s="5">
+        <v>5</v>
+      </c>
+      <c r="G23" s="5">
         <f t="shared" si="0"/>
         <v>4.2309999999999999</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A24" s="16" t="s">
+      <c r="H23" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A24" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B24" s="16" t="s">
+      <c r="B24" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C24" s="18">
+      <c r="C24" s="5">
         <v>4.09</v>
       </c>
-      <c r="D24" s="18">
-        <v>5</v>
-      </c>
-      <c r="E24" s="18">
-        <v>5</v>
-      </c>
-      <c r="F24" s="18">
-        <v>0</v>
-      </c>
-      <c r="G24" s="18">
+      <c r="D24" s="5">
+        <v>5</v>
+      </c>
+      <c r="E24" s="5">
+        <v>5</v>
+      </c>
+      <c r="F24" s="5">
+        <v>0</v>
+      </c>
+      <c r="G24" s="5">
         <f t="shared" si="0"/>
         <v>3.8860000000000001</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A25" s="16" t="s">
+      <c r="H24" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A25" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B25" s="16" t="s">
+      <c r="B25" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C25" s="18">
-        <v>0</v>
-      </c>
-      <c r="D25" s="18">
-        <v>0</v>
-      </c>
-      <c r="E25" s="18">
-        <v>0</v>
-      </c>
-      <c r="F25" s="18">
-        <v>0</v>
-      </c>
-      <c r="G25" s="18">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A26" s="16" t="s">
+      <c r="C25" s="5">
+        <v>0</v>
+      </c>
+      <c r="D25" s="5">
+        <v>0</v>
+      </c>
+      <c r="E25" s="5">
+        <v>0</v>
+      </c>
+      <c r="F25" s="5">
+        <v>0</v>
+      </c>
+      <c r="G25" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H25" s="22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A26" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B26" s="16" t="s">
+      <c r="B26" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C26" s="18">
+      <c r="C26" s="5">
         <v>3.18</v>
       </c>
-      <c r="D26" s="18">
+      <c r="D26" s="5">
         <v>4.38</v>
       </c>
-      <c r="E26" s="18">
-        <v>5</v>
-      </c>
-      <c r="F26" s="18">
-        <v>5</v>
-      </c>
-      <c r="G26" s="18">
+      <c r="E26" s="5">
+        <v>5</v>
+      </c>
+      <c r="F26" s="5">
+        <v>5</v>
+      </c>
+      <c r="G26" s="5">
         <f t="shared" si="0"/>
         <v>4.0860000000000003</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A27" s="16" t="s">
+      <c r="H26" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A27" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B27" s="16" t="s">
+      <c r="B27" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="18">
+      <c r="C27" s="5">
         <v>3.18</v>
       </c>
-      <c r="D27" s="18">
+      <c r="D27" s="5">
         <v>4.82</v>
       </c>
-      <c r="E27" s="18">
-        <v>5</v>
-      </c>
-      <c r="F27" s="18">
-        <v>5</v>
-      </c>
-      <c r="G27" s="18">
+      <c r="E27" s="5">
+        <v>5</v>
+      </c>
+      <c r="F27" s="5">
+        <v>5</v>
+      </c>
+      <c r="G27" s="5">
         <f t="shared" si="0"/>
         <v>4.218</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A28" s="16" t="s">
+      <c r="H27" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A28" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B28" s="16" t="s">
+      <c r="B28" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C28" s="18">
+      <c r="C28" s="5">
         <v>2.0499999999999998</v>
       </c>
-      <c r="D28" s="18">
-        <v>0</v>
-      </c>
-      <c r="E28" s="18">
-        <v>0</v>
-      </c>
-      <c r="F28" s="18">
+      <c r="D28" s="5">
+        <v>0</v>
+      </c>
+      <c r="E28" s="5">
+        <v>0</v>
+      </c>
+      <c r="F28" s="5">
         <v>4.7</v>
       </c>
-      <c r="G28" s="18">
+      <c r="G28" s="5">
         <f t="shared" si="0"/>
         <v>1.5249999999999999</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A29" s="16" t="s">
+      <c r="H28" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A29" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B29" s="16" t="s">
+      <c r="B29" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C29" s="18">
+      <c r="C29" s="5">
         <v>3.18</v>
       </c>
-      <c r="D29" s="18">
+      <c r="D29" s="5">
         <v>3.97</v>
       </c>
-      <c r="E29" s="18">
-        <v>5</v>
-      </c>
-      <c r="F29" s="18">
-        <v>0</v>
-      </c>
-      <c r="G29" s="18">
+      <c r="E29" s="5">
+        <v>5</v>
+      </c>
+      <c r="F29" s="5">
+        <v>0</v>
+      </c>
+      <c r="G29" s="5">
         <f t="shared" si="0"/>
         <v>3.2130000000000001</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A30" s="16" t="s">
+      <c r="H29" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A30" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B30" s="16" t="s">
+      <c r="B30" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C30" s="18">
+      <c r="C30" s="5">
         <v>0.91</v>
       </c>
-      <c r="D30" s="18">
+      <c r="D30" s="5">
         <v>2.66</v>
       </c>
-      <c r="E30" s="18">
-        <v>0</v>
-      </c>
-      <c r="F30" s="18">
-        <v>5</v>
-      </c>
-      <c r="G30" s="18">
+      <c r="E30" s="5">
+        <v>0</v>
+      </c>
+      <c r="F30" s="5">
+        <v>5</v>
+      </c>
+      <c r="G30" s="5">
         <f t="shared" si="0"/>
         <v>1.9120000000000001</v>
+      </c>
+      <c r="H30" s="22">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>